<commit_message>
Add 3_Logical Functions | IF, IFS & update 2_functions, readme file
</commit_message>
<xml_diff>
--- a/2_Formulas_Functions/2_Functions.xlsx
+++ b/2_Formulas_Functions/2_Functions.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7456b23f02075ab8/Documents/Excel LUKE/2_Formulas_Functions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="8_{7AC54B36-9D9E-4574-9B35-E540224EAB9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F75A0C9-06D2-4DB7-AD37-7CB71AB24415}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="8_{7AC54B36-9D9E-4574-9B35-E540224EAB9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{556A78FF-D988-48BA-9E3C-2209B680C706}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{6B78DF1B-62F5-4BE0-BA81-9C8917EAF48C}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="2" r:id="rId1"/>
+    <sheet name="Errors" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,8 +34,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="49">
   <si>
     <t>Job Title</t>
   </si>
@@ -130,6 +153,57 @@
   </si>
   <si>
     <t>Meets Goals Count</t>
+  </si>
+  <si>
+    <t>Error Type</t>
+  </si>
+  <si>
+    <t>Formula</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>=1/0</t>
+  </si>
+  <si>
+    <t>The formula is trying to divide by zero</t>
+  </si>
+  <si>
+    <t>=B4 + "text"</t>
+  </si>
+  <si>
+    <t>The formula includes an argument of the wrong type</t>
+  </si>
+  <si>
+    <t>=#REF!</t>
+  </si>
+  <si>
+    <t>The formula refers to a cell that isn’t valid (usually deleted cell)</t>
+  </si>
+  <si>
+    <t>=COUNTT(A3:A9)</t>
+  </si>
+  <si>
+    <t>The formula uses a name that Excel doesn’t recognize</t>
+  </si>
+  <si>
+    <t>=VLOOKUP("Value", A1:A10, 2, FALSE)</t>
+  </si>
+  <si>
+    <t>The formula is referring to a cell whose data isn’t available</t>
+  </si>
+  <si>
+    <t>=SQRT(-1)</t>
+  </si>
+  <si>
+    <t>There is a problem with the value in the formula</t>
+  </si>
+  <si>
+    <t>=SUM(A1:A10 B1:B10)</t>
+  </si>
+  <si>
+    <t>The formula is trying to use an intersection of two ranges that don’t intersect</t>
   </si>
 </sst>
 </file>
@@ -139,7 +213,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -148,6 +222,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -456,66 +538,72 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1582,4 +1670,115 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{101A623D-18D4-4206-876C-17FE72BDDDBB}">
+  <dimension ref="B2:D9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="2.109375" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" customWidth="1"/>
+    <col min="3" max="3" width="31.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="60.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B2" s="33" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="33" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="33" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B3" s="34" t="e">
+        <f>1/0</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C3" s="35" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="34" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B4" s="34" t="e">
+        <f>A4 + "text"</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="C4" s="35" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="34" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B5" s="36" t="e">
+        <f>#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="C5" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="34" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B6" s="36" t="e" cm="1">
+        <f t="array" aca="1" ref="B6" ca="1">COUNTT(A3:A9)</f>
+        <v>#NAME?</v>
+      </c>
+      <c r="C6" s="35" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="34" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B7" s="34" t="e">
+        <f>VLOOKUP("Value", A1:A10, 2, FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C7" s="35" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="34" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B8" s="34" t="e">
+        <f>SQRT(-1)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="C8" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" s="34" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B9" s="34" t="e">
+        <f>SUM(A1:A10 C1:C10)</f>
+        <v>#NULL!</v>
+      </c>
+      <c r="C9" s="35" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" s="34" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>